<commit_message>
added Session 8 PPTX and RMarkdown notebooks for sessions 6 through 8
</commit_message>
<xml_diff>
--- a/sesion-06/Laboratorio_S06.xlsx
+++ b/sesion-06/Laboratorio_S06.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="P1" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="P2" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Matriz de evidencia" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Fuente P3" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Matriz de evidencia" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="134">
   <si>
     <t xml:space="preserve">Laboratorio Práctico 2 · Sesión 6</t>
   </si>
@@ -49,7 +50,7 @@
     <t xml:space="preserve">Parte 3  ·  10 min</t>
   </si>
   <si>
-    <t xml:space="preserve">Matriz de evidencia. En la hoja «Matriz de evidencia», tomen 3 afirmaciones y llenen su fila: cita textual, ubicación, quién verificó y nivel de confianza.</t>
+    <t xml:space="preserve">Matriz de evidencia. Lee la hoja «Fuente P3» (fragmento de reglas y resumen de la IA), toma 3 afirmaciones y en la hoja «Matriz de evidencia» llena su fila: cita textual, ubicación, quién verificó y nivel de confianza.</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo se usa el archivo</t>
@@ -301,10 +302,91 @@
     <t xml:space="preserve">Rapidísimos, apenas dos horas formado bajo el sol.</t>
   </si>
   <si>
+    <t xml:space="preserve">Parte 3 · Fuente: reglas y resumen de la IA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lee las dos partes. En la hoja «Matriz de evidencia» tomarás 3 afirmaciones del resumen y las rastrearás a este fragmento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fragmento de las Reglas de Operación del PAAC (ficticio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artículo 5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Programa tiene por objeto entregar un apoyo económico a hogares para la compra de alimentos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artículo 8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Son requisitos residir en localidad de alta o muy alta marginación, tener ingreso por debajo de la línea de pobreza extrema y contar con la CURP de la persona titular.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artículo 12.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El monto del apoyo será de 2,000 pesos por hogar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artículo 14.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El apoyo se entregará de manera bimestral.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artículo 19.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las personas beneficiarias deberán asistir a un taller de orientación alimentaria una vez al año.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artículo 23.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Programa operará en las localidades de alta y muy alta marginación de las entidades seleccionadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumen que hizo la IA sobre el programa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El apoyo del Programa se entrega cada dos meses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Programa se dirige a hogares en localidades de alta marginación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El apoyo de 2,000 pesos es suficiente para cubrir la alimentación de un hogar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para recibir el apoyo hay que asistir a un taller cada mes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Programa entrega despensas físicas en centros comunitarios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Algunas afirmaciones se sostienen con el fragmento y otras no. Al llenar la matriz, revisa que la cita diga exactamente lo que la afirmación asegura.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Parte 3 · Matriz de evidencia con trazabilidad</t>
   </si>
   <si>
-    <t xml:space="preserve">Una fila por afirmación. La primera fila es un ejemplo; ustedes llenan las de abajo (ámbar).</t>
+    <t xml:space="preserve">Toma 3 afirmaciones del resumen de la hoja «Fuente P3» y trázalas al fragmento. La primera fila es un ejemplo; llena las de abajo (ámbar).</t>
   </si>
   <si>
     <t xml:space="preserve">Afirmación (como irá en el informe)</t>
@@ -356,7 +438,7 @@
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -536,6 +618,22 @@
       <b val="true"/>
       <sz val="9.5"/>
       <color rgb="FF60707E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12.5"/>
+      <color rgb="FFCB5E2E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10.5"/>
+      <color rgb="FF15293B"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -644,7 +742,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -793,7 +891,27 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -809,7 +927,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1925,6 +2043,155 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="B2:C20"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="84"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="6"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="7"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="37"/>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="38" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="37"/>
+    </row>
+    <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="39" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="40" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="40" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="40" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" s="40" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="39" t="s">
+        <v>116</v>
+      </c>
+      <c r="C18" s="40" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="41" t="s">
+        <v>118</v>
+      </c>
+      <c r="C20" s="41"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B20:C20"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="B2:G14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1939,7 +2206,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="6" t="s">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -1949,7 +2216,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -1958,102 +2225,102 @@
       <c r="G3" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="C5" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>96</v>
-      </c>
-      <c r="E5" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="F5" s="37" t="s">
-        <v>98</v>
-      </c>
-      <c r="G5" s="37" t="s">
-        <v>99</v>
+      <c r="B5" s="42" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>123</v>
+      </c>
+      <c r="E5" s="42" t="s">
+        <v>124</v>
+      </c>
+      <c r="F5" s="42" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="C6" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="39" t="s">
-        <v>103</v>
-      </c>
-      <c r="F6" s="39" t="s">
-        <v>104</v>
-      </c>
-      <c r="G6" s="39" t="s">
-        <v>105</v>
+      <c r="B6" s="43" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" s="44" t="s">
+        <v>129</v>
+      </c>
+      <c r="E6" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="F6" s="44" t="s">
+        <v>131</v>
+      </c>
+      <c r="G6" s="44" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
     </row>
     <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
     </row>
     <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="40"/>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
     </row>
     <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="45"/>
+      <c r="G12" s="45"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="41" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
+      <c r="B14" s="46" t="s">
+        <v>133</v>
+      </c>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>